<commit_message>
feat: Param optimization now also covers.
</commit_message>
<xml_diff>
--- a/experiment/param_optimization_results/gpt-5-nano-2025-08-07_param_optimization_1.xlsx
+++ b/experiment/param_optimization_results/gpt-5-nano-2025-08-07_param_optimization_1.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -427,6 +427,16 @@
           <t>gen_math w/ cs 1 1</t>
         </is>
       </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>gsm  1 1</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>gsm w/ cs 1 1</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -440,6 +450,12 @@
       <c r="C2" t="n">
         <v>1</v>
       </c>
+      <c r="D2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E2" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -453,6 +469,12 @@
       <c r="C3" t="n">
         <v>1</v>
       </c>
+      <c r="D3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -466,6 +488,12 @@
       <c r="C4" t="n">
         <v>1</v>
       </c>
+      <c r="D4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -483,6 +511,16 @@
           <t>gpt-5-nano-2025-08-07</t>
         </is>
       </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>gpt-5-nano-2025-08-07</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>gpt-5-nano-2025-08-07</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -496,6 +534,12 @@
       <c r="C6" t="n">
         <v>0</v>
       </c>
+      <c r="D6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -509,6 +553,12 @@
       <c r="C7" t="n">
         <v>1</v>
       </c>
+      <c r="D7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -517,11 +567,17 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>16.99</v>
+        <v>17.08</v>
       </c>
       <c r="C8" t="n">
         <v>0.06</v>
       </c>
+      <c r="D8" t="n">
+        <v>6.18</v>
+      </c>
+      <c r="E8" t="n">
+        <v>5.64</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -535,6 +591,12 @@
       <c r="C9" t="n">
         <v>0</v>
       </c>
+      <c r="D9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -552,6 +614,16 @@
           <t>(1.0, 1.0)</t>
         </is>
       </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>(1.0, 1.0)</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>(1.0, 1.0)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -565,6 +637,12 @@
       <c r="C11" t="n">
         <v>0</v>
       </c>
+      <c r="D11" t="n">
+        <v>85</v>
+      </c>
+      <c r="E11" t="n">
+        <v>85</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -578,6 +656,12 @@
       <c r="C12" t="n">
         <v>64</v>
       </c>
+      <c r="D12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -591,6 +675,12 @@
       <c r="C13" t="n">
         <v>0</v>
       </c>
+      <c r="D13" t="n">
+        <v>4.25e-06</v>
+      </c>
+      <c r="E13" t="n">
+        <v>4.25e-06</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -604,6 +694,12 @@
       <c r="C14" t="n">
         <v>3.2e-06</v>
       </c>
+      <c r="D14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -612,10 +708,16 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>1527</v>
+        <v>1822</v>
       </c>
       <c r="C15" t="n">
         <v>0</v>
+      </c>
+      <c r="D15" t="n">
+        <v>458</v>
+      </c>
+      <c r="E15" t="n">
+        <v>464</v>
       </c>
     </row>
     <row r="16">
@@ -630,6 +732,12 @@
       <c r="C16" t="n">
         <v>2818</v>
       </c>
+      <c r="D16" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -638,10 +746,16 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>0.0006108000000000001</v>
+        <v>0.0007288</v>
       </c>
       <c r="C17" t="n">
         <v>0</v>
+      </c>
+      <c r="D17" t="n">
+        <v>0.0001832</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0.0001856</v>
       </c>
     </row>
     <row r="18">
@@ -656,6 +770,12 @@
       <c r="C18" t="n">
         <v>0.0011272</v>
       </c>
+      <c r="D18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -664,10 +784,16 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>0.0006140000000000001</v>
+        <v>0.000732</v>
       </c>
       <c r="C19" t="n">
         <v>0</v>
+      </c>
+      <c r="D19" t="n">
+        <v>0.00018745</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0.00018985</v>
       </c>
     </row>
     <row r="20">
@@ -682,18 +808,30 @@
       <c r="C20" t="n">
         <v>0.0011304</v>
       </c>
+      <c r="D20" t="n">
+        <v>0</v>
+      </c>
+      <c r="E20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>total_cost ($)</t>
+          <t>cost_paid_w/o_cs ($)</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>0.0006140000000000001</v>
+        <v>0.000732</v>
       </c>
       <c r="C21" t="n">
-        <v>-0.0011304</v>
+        <v>0.0011304</v>
+      </c>
+      <c r="D21" t="n">
+        <v>0.00018745</v>
+      </c>
+      <c r="E21" t="n">
+        <v>0.00018985</v>
       </c>
     </row>
   </sheetData>

</xml_diff>